<commit_message>
Análisis de estadísticas: guía de videos, programa y Excel conectado
- marca/guia-videos.md: qué mide cada número, reglas para sacar conclusiones,
  reglas vigentes, hipótesis por probar y registro de análisis.
- herramientas/analisis/estadisticas.py: importa datos de Metricool (Reels de
  Instagram y videos de TikTok), guarda lecturas a 48 h y 7 días, leads y tabla.
- analisis/videos.json: ficha de los 5 videos para comparar variables.
- build.py: la pestaña Resultados se llena sola con analisis/estadisticas.json.
- CLAUDE.md: pasos para crear videos y para analizar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013nTNBrNgFLGCMuMdkBmq2A
</commit_message>
<xml_diff>
--- a/marca/lumen-calendario-publicaciones.xlsx
+++ b/marca/lumen-calendario-publicaciones.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -73,11 +74,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="000F172A"/>
       <sz val="10"/>
@@ -101,11 +97,16 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -119,7 +120,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
+        <fgColor rgb="00E6F7F4"/>
       </patternFill>
     </fill>
     <fill>
@@ -130,6 +131,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00CCFBF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -159,24 +165,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,26 +212,32 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -617,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -711,72 +723,83 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>Resultados!E15</f>
+        <f>Resultados!F15</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Mensajes recibidos</t>
+          <t>Seguidores ganados (48 h)</t>
         </is>
       </c>
       <c r="B11" s="5">
-        <f>Resultados!M15</f>
+        <f>Resultados!Q15</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>Mensajes recibidos</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>Resultados!R15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>Clientes que cotizaron</t>
         </is>
       </c>
-      <c r="B12" s="5">
-        <f>Resultados!N15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="B13" s="5">
+        <f>Resultados!S15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Créditos de voz (ElevenLabs Starter)</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Créditos disponibles</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>38848</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Costo por video (aprox.)</t>
+          <t>Créditos disponibles</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>400</v>
+        <v>38848</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>Costo por video (aprox.)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
           <t>Videos que alcanzan</t>
         </is>
       </c>
-      <c r="B17" s="9">
-        <f>IFERROR(INT(B15/B16),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="B18" s="9">
+        <f>IFERROR(INT(B16/B17),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Fuente: tu cuenta de ElevenLabs (15/10/2026). Voz: Diego (desde el video 4). Los créditos se renuevan cada mes.</t>
         </is>
@@ -1479,7 +1502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1489,13 +1512,18 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1508,7 +1536,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Celdas amarillas: escribe los números de Metricool o de la app. Las columnas grises se calculan solas.</t>
+          <t>Claude llena esta pestaña con los datos de Metricool (a las 48 h y a los 7 días de cada video). Las columnas grises se calculan solas.</t>
         </is>
       </c>
     </row>
@@ -1535,50 +1563,75 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
+          <t>Horas publicado</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
           <t>Vistas</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Alcance</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Vio +3 s (IG) / completo (TT)</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>% visto</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>Tiempo medio (s)</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>Me gusta</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr">
         <is>
           <t>Comentarios</t>
         </is>
       </c>
-      <c r="I4" s="10" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>Guardados</t>
         </is>
       </c>
-      <c r="J4" s="10" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr">
         <is>
           <t>Compartidos</t>
         </is>
       </c>
-      <c r="K4" s="10" t="inlineStr">
+      <c r="O4" s="10" t="inlineStr">
         <is>
           <t>Interacciones</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Tasa de interacción</t>
         </is>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>Seguidores 48 h</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Mensajes recibidos</t>
         </is>
       </c>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="S4" s="10" t="inlineStr">
         <is>
           <t>Clientes que cotizaron</t>
         </is>
@@ -1601,22 +1654,27 @@
         <f>Calendario!F5</f>
         <v/>
       </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="18">
-        <f>IF(COUNT(G5:J5)=0,"",SUM(G5:J5))</f>
-        <v/>
-      </c>
-      <c r="L5" s="19">
-        <f>IFERROR(IF(F5="","",K5/F5),"")</f>
-        <v/>
-      </c>
-      <c r="M5" s="20" t="n"/>
-      <c r="N5" s="20" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="19" t="n"/>
+      <c r="H5" s="20" t="n"/>
+      <c r="I5" s="20" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="19" t="n"/>
+      <c r="L5" s="19" t="n"/>
+      <c r="M5" s="19" t="n"/>
+      <c r="N5" s="19" t="n"/>
+      <c r="O5" s="21">
+        <f>IF(COUNT(K5:N5)=0,"",SUM(K5:N5))</f>
+        <v/>
+      </c>
+      <c r="P5" s="22">
+        <f>IFERROR(IF(G5="","",O5/G5),"")</f>
+        <v/>
+      </c>
+      <c r="Q5" s="19" t="n"/>
+      <c r="R5" s="19" t="n"/>
+      <c r="S5" s="19" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="16">
@@ -1635,22 +1693,27 @@
         <f>Calendario!F6</f>
         <v/>
       </c>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="21" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="18">
-        <f>IF(COUNT(G6:J6)=0,"",SUM(G6:J6))</f>
-        <v/>
-      </c>
-      <c r="L6" s="19">
-        <f>IFERROR(IF(F6="","",K6/F6),"")</f>
-        <v/>
-      </c>
-      <c r="M6" s="20" t="n"/>
-      <c r="N6" s="20" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+      <c r="H6" s="20" t="n"/>
+      <c r="I6" s="20" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="19" t="n"/>
+      <c r="L6" s="19" t="n"/>
+      <c r="M6" s="21" t="n"/>
+      <c r="N6" s="19" t="n"/>
+      <c r="O6" s="21">
+        <f>IF(COUNT(K6:N6)=0,"",SUM(K6:N6))</f>
+        <v/>
+      </c>
+      <c r="P6" s="22">
+        <f>IFERROR(IF(G6="","",O6/G6),"")</f>
+        <v/>
+      </c>
+      <c r="Q6" s="19" t="n"/>
+      <c r="R6" s="19" t="n"/>
+      <c r="S6" s="19" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="16">
@@ -1669,22 +1732,27 @@
         <f>Calendario!F7</f>
         <v/>
       </c>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="18">
-        <f>IF(COUNT(G7:J7)=0,"",SUM(G7:J7))</f>
-        <v/>
-      </c>
-      <c r="L7" s="19">
-        <f>IFERROR(IF(F7="","",K7/F7),"")</f>
-        <v/>
-      </c>
-      <c r="M7" s="20" t="n"/>
-      <c r="N7" s="20" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="20" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="19" t="n"/>
+      <c r="L7" s="19" t="n"/>
+      <c r="M7" s="19" t="n"/>
+      <c r="N7" s="19" t="n"/>
+      <c r="O7" s="21">
+        <f>IF(COUNT(K7:N7)=0,"",SUM(K7:N7))</f>
+        <v/>
+      </c>
+      <c r="P7" s="22">
+        <f>IFERROR(IF(G7="","",O7/G7),"")</f>
+        <v/>
+      </c>
+      <c r="Q7" s="19" t="n"/>
+      <c r="R7" s="19" t="n"/>
+      <c r="S7" s="19" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="16">
@@ -1703,22 +1771,27 @@
         <f>Calendario!F8</f>
         <v/>
       </c>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="21" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="18">
-        <f>IF(COUNT(G8:J8)=0,"",SUM(G8:J8))</f>
-        <v/>
-      </c>
-      <c r="L8" s="19">
-        <f>IFERROR(IF(F8="","",K8/F8),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="20" t="n"/>
-      <c r="N8" s="20" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="20" t="n"/>
+      <c r="I8" s="20" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="21" t="n"/>
+      <c r="N8" s="19" t="n"/>
+      <c r="O8" s="21">
+        <f>IF(COUNT(K8:N8)=0,"",SUM(K8:N8))</f>
+        <v/>
+      </c>
+      <c r="P8" s="22">
+        <f>IFERROR(IF(G8="","",O8/G8),"")</f>
+        <v/>
+      </c>
+      <c r="Q8" s="19" t="n"/>
+      <c r="R8" s="19" t="n"/>
+      <c r="S8" s="19" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="16">
@@ -1737,22 +1810,27 @@
         <f>Calendario!F9</f>
         <v/>
       </c>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="18">
-        <f>IF(COUNT(G9:J9)=0,"",SUM(G9:J9))</f>
-        <v/>
-      </c>
-      <c r="L9" s="19">
-        <f>IFERROR(IF(F9="","",K9/F9),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="20" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="20" t="n"/>
+      <c r="I9" s="20" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="19" t="n"/>
+      <c r="L9" s="19" t="n"/>
+      <c r="M9" s="19" t="n"/>
+      <c r="N9" s="19" t="n"/>
+      <c r="O9" s="21">
+        <f>IF(COUNT(K9:N9)=0,"",SUM(K9:N9))</f>
+        <v/>
+      </c>
+      <c r="P9" s="22">
+        <f>IFERROR(IF(G9="","",O9/G9),"")</f>
+        <v/>
+      </c>
+      <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="16">
@@ -1771,22 +1849,27 @@
         <f>Calendario!F10</f>
         <v/>
       </c>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="21" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="18">
-        <f>IF(COUNT(G10:J10)=0,"",SUM(G10:J10))</f>
-        <v/>
-      </c>
-      <c r="L10" s="19">
-        <f>IFERROR(IF(F10="","",K10/F10),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="20" t="n"/>
-      <c r="N10" s="20" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="20" t="n"/>
+      <c r="I10" s="20" t="n"/>
+      <c r="J10" s="18" t="n"/>
+      <c r="K10" s="19" t="n"/>
+      <c r="L10" s="19" t="n"/>
+      <c r="M10" s="21" t="n"/>
+      <c r="N10" s="19" t="n"/>
+      <c r="O10" s="21">
+        <f>IF(COUNT(K10:N10)=0,"",SUM(K10:N10))</f>
+        <v/>
+      </c>
+      <c r="P10" s="22">
+        <f>IFERROR(IF(G10="","",O10/G10),"")</f>
+        <v/>
+      </c>
+      <c r="Q10" s="19" t="n"/>
+      <c r="R10" s="19" t="n"/>
+      <c r="S10" s="19" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="16">
@@ -1805,22 +1888,27 @@
         <f>Calendario!F11</f>
         <v/>
       </c>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="18">
-        <f>IF(COUNT(G11:J11)=0,"",SUM(G11:J11))</f>
-        <v/>
-      </c>
-      <c r="L11" s="19">
-        <f>IFERROR(IF(F11="","",K11/F11),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="20" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
+      <c r="H11" s="20" t="n"/>
+      <c r="I11" s="20" t="n"/>
+      <c r="J11" s="18" t="n"/>
+      <c r="K11" s="19" t="n"/>
+      <c r="L11" s="19" t="n"/>
+      <c r="M11" s="19" t="n"/>
+      <c r="N11" s="19" t="n"/>
+      <c r="O11" s="21">
+        <f>IF(COUNT(K11:N11)=0,"",SUM(K11:N11))</f>
+        <v/>
+      </c>
+      <c r="P11" s="22">
+        <f>IFERROR(IF(G11="","",O11/G11),"")</f>
+        <v/>
+      </c>
+      <c r="Q11" s="19" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="16">
@@ -1839,22 +1927,27 @@
         <f>Calendario!F12</f>
         <v/>
       </c>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="18">
-        <f>IF(COUNT(G12:J12)=0,"",SUM(G12:J12))</f>
-        <v/>
-      </c>
-      <c r="L12" s="19">
-        <f>IFERROR(IF(F12="","",K12/F12),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="20" t="n"/>
-      <c r="N12" s="20" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
+      <c r="H12" s="20" t="n"/>
+      <c r="I12" s="20" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="21" t="n"/>
+      <c r="N12" s="19" t="n"/>
+      <c r="O12" s="21">
+        <f>IF(COUNT(K12:N12)=0,"",SUM(K12:N12))</f>
+        <v/>
+      </c>
+      <c r="P12" s="22">
+        <f>IFERROR(IF(G12="","",O12/G12),"")</f>
+        <v/>
+      </c>
+      <c r="Q12" s="19" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="16">
@@ -1873,22 +1966,27 @@
         <f>Calendario!F13</f>
         <v/>
       </c>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="18">
-        <f>IF(COUNT(G13:J13)=0,"",SUM(G13:J13))</f>
-        <v/>
-      </c>
-      <c r="L13" s="19">
-        <f>IFERROR(IF(F13="","",K13/F13),"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="20" t="n"/>
-      <c r="N13" s="20" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="20" t="n"/>
+      <c r="I13" s="20" t="n"/>
+      <c r="J13" s="18" t="n"/>
+      <c r="K13" s="19" t="n"/>
+      <c r="L13" s="19" t="n"/>
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="19" t="n"/>
+      <c r="O13" s="21">
+        <f>IF(COUNT(K13:N13)=0,"",SUM(K13:N13))</f>
+        <v/>
+      </c>
+      <c r="P13" s="22">
+        <f>IFERROR(IF(G13="","",O13/G13),"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="16">
@@ -1907,32 +2005,33 @@
         <f>Calendario!F14</f>
         <v/>
       </c>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="8" t="n"/>
-      <c r="I14" s="21" t="n"/>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="18">
-        <f>IF(COUNT(G14:J14)=0,"",SUM(G14:J14))</f>
-        <v/>
-      </c>
-      <c r="L14" s="19">
-        <f>IFERROR(IF(F14="","",K14/F14),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="20" t="n"/>
-      <c r="N14" s="20" t="n"/>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="20" t="n"/>
+      <c r="I14" s="20" t="n"/>
+      <c r="J14" s="18" t="n"/>
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="21" t="n"/>
+      <c r="N14" s="19" t="n"/>
+      <c r="O14" s="21">
+        <f>IF(COUNT(K14:N14)=0,"",SUM(K14:N14))</f>
+        <v/>
+      </c>
+      <c r="P14" s="22">
+        <f>IFERROR(IF(G14="","",O14/G14),"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="22" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E15" s="5">
-        <f>SUM(E5:E14)</f>
-        <v/>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Total / promedio</t>
+        </is>
       </c>
       <c r="F15" s="5">
         <f>SUM(F5:F14)</f>
@@ -1942,24 +2041,24 @@
         <f>SUM(G5:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="5">
-        <f>SUM(H5:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="5">
-        <f>SUM(I5:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="5">
-        <f>SUM(J5:J14)</f>
+      <c r="H15" s="24">
+        <f>IFERROR(AVERAGE(H5:H14),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="24">
+        <f>IFERROR(AVERAGE(I5:I14),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="25">
+        <f>IFERROR(AVERAGE(J5:J14),"")</f>
         <v/>
       </c>
       <c r="K15" s="5">
         <f>SUM(K5:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="23">
-        <f>IFERROR(IF(F15=0,"",K15/F15),"")</f>
+      <c r="L15" s="5">
+        <f>SUM(L5:L14)</f>
         <v/>
       </c>
       <c r="M15" s="5">
@@ -1970,39 +2069,73 @@
         <f>SUM(N5:N14)</f>
         <v/>
       </c>
+      <c r="O15" s="5">
+        <f>SUM(O5:O14)</f>
+        <v/>
+      </c>
+      <c r="P15" s="24">
+        <f>IFERROR(IF(G15=0,"",O15/G15),"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="5">
+        <f>SUM(Q5:Q14)</f>
+        <v/>
+      </c>
+      <c r="R15" s="5">
+        <f>SUM(R5:R14)</f>
+        <v/>
+      </c>
+      <c r="S15" s="5">
+        <f>SUM(S5:S14)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="25" t="inlineStr">
-        <is>
-          <t>• Metricool todavía no muestra estadísticas (cuenta conectada hoy); suelen aparecer en unas 24 horas.</t>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>• Última lectura de Metricool: todavía sin datos (la cuenta se conectó el 15/10/2026).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="25" t="inlineStr">
-        <is>
-          <t>• Interacciones = Me gusta + Comentarios + Guardados + Compartidos. Tasa de interacción = Interacciones ÷ Alcance.</t>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>• Vio +3 s (Instagram): % de vistas que pasaron de los 3 primeros segundos; mide el gancho. Vio completo (TikTok): % que vio todo el video.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="25" t="inlineStr">
-        <is>
-          <t>• TikTok no informa 'Guardados' por Metricool, por eso esa celda está en gris.</t>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>• % visto: parte del video que se ve en promedio. Interacciones = Me gusta + Comentarios + Guardados + Compartidos. Tasa = Interacciones ÷ Alcance.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="25" t="inlineStr">
-        <is>
-          <t>• Mensajes recibidos y Clientes que cotizaron: llévalos tú a mano; son los números que de verdad importan para vender.</t>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>• Seguidores 48 h: ganados el día de la publicación y el siguiente. TikTok no informa 'Guardados' por Metricool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>• Mensajes y clientes: cuéntale a Claude cuando te escriba alguien y de qué video viene; son los números que de verdad importan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>• Lo aprendido de cada video está en marca/guia-videos.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Video 6 programado; paso a 1 video diario y temas aprobados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014uTc5G6VvPKerEinMqYdQX
</commit_message>
<xml_diff>
--- a/marca/lumen-calendario-publicaciones.xlsx
+++ b/marca/lumen-calendario-publicaciones.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calendario'!$A$4:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calendario'!$A$4:$K$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>Resultados!F15</f>
+        <f>Resultados!F17</f>
         <v/>
       </c>
     </row>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>Resultados!Q15</f>
+        <f>Resultados!Q17</f>
         <v/>
       </c>
     </row>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>Resultados!R15</f>
+        <f>Resultados!R17</f>
         <v/>
       </c>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>Resultados!S15</f>
+        <f>Resultados!S17</f>
         <v/>
       </c>
     </row>
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1473,9 +1473,121 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>3 errores que espantan clientes</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>vie 16/10/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>12:15 pm</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Programado</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Se genera al publicarse</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Una web lenta no solo pierde visitas: Google también la muestra más abajo en los resultados 🔎
+Y el botón de WhatsApp no es un detalle: es el camino más corto entre "me interesa" y "quiero comprar" 💬
+¿Cuál de estos 3 errores has visto más en las webs de negocios? Te leo en los comentarios 👇 o escríbeme por WhatsApp desde el enlace de mi biografía.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>#diseñoweb #paginasweb #webdesign #emprendedoresvenezolanos #aragua #maracay #venezuela #negociosvenezuela #marketingdigital #emprendimiento</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>lumen-reel-06-errores-que-espantan-clientes.mp4</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>Título (seg. 1,8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>3 errores que espantan clientes</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>vie 16/10/2026</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>12:15 pm</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Programado</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Se genera al publicarse</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Una web lenta también aparece más abajo en Google 🔎 y el botón de WhatsApp es el camino más corto entre "me interesa" y "quiero comprar" 💬 ¿Cuál de estos 3 errores has visto más? Cuéntame en los comentarios o escríbeme por mensaje directo</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>#diseñoweb #paginasweb #emprendedoresvenezolanos #venezuela #negocios</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>lumen-reel-06-errores-que-espantan-clientes-tiktok.mp4</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>Primer fotograma</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K14"/>
-  <conditionalFormatting sqref="F5:F14">
+  <autoFilter ref="A4:K16"/>
+  <conditionalFormatting sqref="F5:F16">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="Publicado"</formula>
     </cfRule>
@@ -1484,7 +1596,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Publicado,Programado,Pendiente,Borrador"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1502,7 +1614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S23"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2027,113 +2139,191 @@
       <c r="R14" s="19" t="n"/>
       <c r="S14" s="19" t="n"/>
     </row>
-    <row r="15">
-      <c r="B15" s="23" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="16">
+        <f>Calendario!A15</f>
+        <v/>
+      </c>
+      <c r="B15" s="17">
+        <f>Calendario!B15</f>
+        <v/>
+      </c>
+      <c r="C15" s="16">
+        <f>Calendario!E15</f>
+        <v/>
+      </c>
+      <c r="D15" s="16">
+        <f>Calendario!F15</f>
+        <v/>
+      </c>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="20" t="n"/>
+      <c r="I15" s="20" t="n"/>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="19" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="19" t="n"/>
+      <c r="N15" s="19" t="n"/>
+      <c r="O15" s="21">
+        <f>IF(COUNT(K15:N15)=0,"",SUM(K15:N15))</f>
+        <v/>
+      </c>
+      <c r="P15" s="22">
+        <f>IFERROR(IF(G15="","",O15/G15),"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="16">
+        <f>Calendario!A16</f>
+        <v/>
+      </c>
+      <c r="B16" s="17">
+        <f>Calendario!B16</f>
+        <v/>
+      </c>
+      <c r="C16" s="16">
+        <f>Calendario!E16</f>
+        <v/>
+      </c>
+      <c r="D16" s="16">
+        <f>Calendario!F16</f>
+        <v/>
+      </c>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="20" t="n"/>
+      <c r="I16" s="20" t="n"/>
+      <c r="J16" s="18" t="n"/>
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19" t="n"/>
+      <c r="M16" s="21" t="n"/>
+      <c r="N16" s="19" t="n"/>
+      <c r="O16" s="21">
+        <f>IF(COUNT(K16:N16)=0,"",SUM(K16:N16))</f>
+        <v/>
+      </c>
+      <c r="P16" s="22">
+        <f>IFERROR(IF(G16="","",O16/G16),"")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>Total / promedio</t>
         </is>
       </c>
-      <c r="F15" s="5">
-        <f>SUM(F5:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="5">
-        <f>SUM(G5:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="24">
-        <f>IFERROR(AVERAGE(H5:H14),"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="24">
-        <f>IFERROR(AVERAGE(I5:I14),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="25">
-        <f>IFERROR(AVERAGE(J5:J14),"")</f>
-        <v/>
-      </c>
-      <c r="K15" s="5">
-        <f>SUM(K5:K14)</f>
-        <v/>
-      </c>
-      <c r="L15" s="5">
-        <f>SUM(L5:L14)</f>
-        <v/>
-      </c>
-      <c r="M15" s="5">
-        <f>SUM(M5:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="5">
-        <f>SUM(N5:N14)</f>
-        <v/>
-      </c>
-      <c r="O15" s="5">
-        <f>SUM(O5:O14)</f>
-        <v/>
-      </c>
-      <c r="P15" s="24">
-        <f>IFERROR(IF(G15=0,"",O15/G15),"")</f>
-        <v/>
-      </c>
-      <c r="Q15" s="5">
-        <f>SUM(Q5:Q14)</f>
-        <v/>
-      </c>
-      <c r="R15" s="5">
-        <f>SUM(R5:R14)</f>
-        <v/>
-      </c>
-      <c r="S15" s="5">
-        <f>SUM(S5:S14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="26" t="inlineStr">
+      <c r="F17" s="5">
+        <f>SUM(F5:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>SUM(G5:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="24">
+        <f>IFERROR(AVERAGE(H5:H16),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="24">
+        <f>IFERROR(AVERAGE(I5:I16),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="25">
+        <f>IFERROR(AVERAGE(J5:J16),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="5">
+        <f>SUM(K5:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="5">
+        <f>SUM(L5:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="5">
+        <f>SUM(M5:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="5">
+        <f>SUM(N5:N16)</f>
+        <v/>
+      </c>
+      <c r="O17" s="5">
+        <f>SUM(O5:O16)</f>
+        <v/>
+      </c>
+      <c r="P17" s="24">
+        <f>IFERROR(IF(G17=0,"",O17/G17),"")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="5">
+        <f>SUM(Q5:Q16)</f>
+        <v/>
+      </c>
+      <c r="R17" s="5">
+        <f>SUM(R5:R16)</f>
+        <v/>
+      </c>
+      <c r="S17" s="5">
+        <f>SUM(S5:S16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Notas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>• Última lectura de Metricool: todavía sin datos (la cuenta se conectó el 15/10/2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="27" t="inlineStr">
-        <is>
-          <t>• Vio +3 s (Instagram): % de vistas que pasaron de los 3 primeros segundos; mide el gancho. Vio completo (TikTok): % que vio todo el video.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>• % visto: parte del video que se ve en promedio. Interacciones = Me gusta + Comentarios + Guardados + Compartidos. Tasa = Interacciones ÷ Alcance.</t>
+          <t>• Última lectura de Metricool: todavía sin datos (la cuenta se conectó el 15/10/2026).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>• Seguidores 48 h: ganados el día de la publicación y el siguiente. TikTok no informa 'Guardados' por Metricool.</t>
+          <t>• Vio +3 s (Instagram): % de vistas que pasaron de los 3 primeros segundos; mide el gancho. Vio completo (TikTok): % que vio todo el video.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>• Mensajes y clientes: cuéntale a Claude cuando te escriba alguien y de qué video viene; son los números que de verdad importan.</t>
+          <t>• % visto: parte del video que se ve en promedio. Interacciones = Me gusta + Comentarios + Guardados + Compartidos. Tasa = Interacciones ÷ Alcance.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>• Seguidores 48 h: ganados el día de la publicación y el siguiente. TikTok no informa 'Guardados' por Metricool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>• Mensajes y clientes: cuéntale a Claude cuando te escriba alguien y de qué video viene; son los números que de verdad importan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>• Lo aprendido de cada video está en marca/guia-videos.md.</t>
         </is>

</xml_diff>

<commit_message>
Video 6 TikTok reprogramado con portada a las 6:00 pm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014uTc5G6VvPKerEinMqYdQX
</commit_message>
<xml_diff>
--- a/marca/lumen-calendario-publicaciones.xlsx
+++ b/marca/lumen-calendario-publicaciones.xlsx
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>12:15 pm</t>
+          <t>6:00 pm</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>lumen-reel-06-errores-que-espantan-clientes-tiktok.mp4</t>
+          <t>lumen-reel-06-errores-que-espantan-clientes-tiktok-portada.mp4</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">

</xml_diff>